<commit_message>
fix(sanity-check): label the Plan and Var to plan columns in the dirty fixture
The columns carrying the Hygiene case were written without headers, so the
typed-but-agreeing total sat in an unlabelled formula column. A run could
reasonably have read the unlabelled pair as a defect in its own right, which
would have tested the wrong thing.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/sanity-check/skills/sanity-check/evals/pack-2026-11-dirty.xlsx
+++ b/plugins/sanity-check/skills/sanity-check/evals/pack-2026-11-dirty.xlsx
@@ -485,6 +485,16 @@
           <t>Headcount</t>
         </is>
       </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Plan (£000s)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Var to plan</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">

</xml_diff>